<commit_message>
CAMBIOS EN SCRIPT PARA GENERRAR INSERT BASES DE ESQUEMA SEGURIDAD
</commit_message>
<xml_diff>
--- a/BD SEGURIDAD.xlsx
+++ b/BD SEGURIDAD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\Code Generator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Datos GNOTO\Code Source\CodeGenerator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03327AB4-8170-41FC-B2B8-C73BDBC904FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E1CEC47-6B4C-4663-94CD-185609A949CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{C9EA7287-3C78-415A-956B-26A527F8C3B3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C9EA7287-3C78-415A-956B-26A527F8C3B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
   <si>
     <t>Id</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>/Metrica</t>
+  </si>
+  <si>
+    <t>INDEX</t>
   </si>
 </sst>
 </file>
@@ -346,14 +349,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -673,26 +674,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25A81F2-8E17-4EB3-9B5C-756069B73C22}">
   <dimension ref="B1:L57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.109375" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.21875" customWidth="1"/>
-    <col min="8" max="8" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.28515625" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="2:12" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
@@ -724,7 +725,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B3" s="1">
         <v>1</v>
       </c>
@@ -741,7 +742,7 @@
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>2</v>
       </c>
@@ -758,7 +759,7 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -769,7 +770,7 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
@@ -777,7 +778,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>0</v>
       </c>
@@ -790,17 +791,17 @@
       <c r="E8" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>1</v>
       </c>
@@ -819,7 +820,7 @@
       </c>
       <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>2</v>
       </c>
@@ -838,7 +839,7 @@
       </c>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -847,12 +848,12 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
         <v>0</v>
       </c>
@@ -874,14 +875,14 @@
       <c r="H15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="I15" s="8" t="s">
+      <c r="I15" s="6" t="s">
         <v>30</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="1">
         <v>1</v>
       </c>
@@ -899,14 +900,14 @@
       <c r="H16" s="1">
         <v>1</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="7">
         <v>1</v>
       </c>
       <c r="J16" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <v>2</v>
       </c>
@@ -924,10 +925,10 @@
       <c r="H17" s="1">
         <v>2</v>
       </c>
-      <c r="I17" s="7"/>
+      <c r="I17" s="5"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <v>3</v>
       </c>
@@ -948,12 +949,12 @@
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>0</v>
       </c>
@@ -985,7 +986,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="1">
         <v>1</v>
       </c>
@@ -1009,7 +1010,7 @@
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B24" s="1">
         <v>2</v>
       </c>
@@ -1033,7 +1034,7 @@
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -1045,12 +1046,12 @@
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B28" s="3" t="s">
         <v>0</v>
       </c>
@@ -1066,11 +1067,11 @@
       <c r="F28" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G28" s="5" t="s">
+      <c r="G28" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B29" s="1">
         <v>1</v>
       </c>
@@ -1078,17 +1079,19 @@
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F29" s="1"/>
       <c r="G29" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B30" s="1">
         <v>2</v>
       </c>
@@ -1096,17 +1099,19 @@
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F30" s="1"/>
+      <c r="F30" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="G30" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B31" s="1">
         <v>2</v>
       </c>
@@ -1114,17 +1119,19 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F31" s="1"/>
+      <c r="F31" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="G31" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B32" s="1">
         <v>3</v>
       </c>
@@ -1132,17 +1139,19 @@
         <v>1</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F32" s="1"/>
+      <c r="F32" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="G32" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B33" s="1">
         <v>4</v>
       </c>
@@ -1150,17 +1159,19 @@
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="F33" s="1"/>
+      <c r="F33" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="G33" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B34" s="1">
         <v>5</v>
       </c>
@@ -1168,58 +1179,64 @@
         <v>2</v>
       </c>
       <c r="D34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E34" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F34" s="1"/>
       <c r="G34" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B35" s="1">
         <v>6</v>
       </c>
       <c r="C35" s="1">
         <v>2</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>55</v>
+      <c r="D35" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="F35" s="1"/>
+      <c r="F35" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="G35" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
         <v>7</v>
       </c>
       <c r="C36" s="1">
         <v>2</v>
       </c>
-      <c r="D36" s="6" t="s">
-        <v>56</v>
+      <c r="D36" s="1" t="s">
+        <v>67</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F36" s="1"/>
+      <c r="F36" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="G36" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B38" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
         <v>22</v>
       </c>
@@ -1230,27 +1247,27 @@
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
     </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
     </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
     </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B45" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B46" s="3" t="s">
         <v>0</v>
       </c>
@@ -1276,7 +1293,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
@@ -1286,7 +1303,7 @@
       <c r="H47" s="1"/>
       <c r="I47" s="1"/>
     </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
@@ -1296,7 +1313,7 @@
       <c r="H48" s="1"/>
       <c r="I48" s="1"/>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
@@ -1306,7 +1323,7 @@
       <c r="H49" s="1"/>
       <c r="I49" s="1"/>
     </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
@@ -1316,12 +1333,12 @@
       <c r="H50" s="1"/>
       <c r="I50" s="1"/>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B53" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B54" s="3" t="s">
         <v>0</v>
       </c>
@@ -1344,7 +1361,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
@@ -1353,7 +1370,7 @@
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
     </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
@@ -1362,7 +1379,7 @@
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
     </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>

</xml_diff>